<commit_message>
Actualización de datos desde Streamlit
</commit_message>
<xml_diff>
--- a/proyectos_v2.xlsx
+++ b/proyectos_v2.xlsx
@@ -3572,10 +3572,10 @@
         <v>145</v>
       </c>
       <c r="G60" t="n">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="H60" t="n">
-        <v>82.65000000000001</v>
+        <v>107.3</v>
       </c>
       <c r="I60" t="inlineStr"/>
       <c r="J60" s="1" t="n">

</xml_diff>